<commit_message>
Update reproducibility materials for PLOS submission
</commit_message>
<xml_diff>
--- a/Variables Chosen.xlsx
+++ b/Variables Chosen.xlsx
@@ -1646,7 +1646,7 @@
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>Energy intensity level of primary energy (MJ/$2017 PPP GDP)_x</t>
+          <t>Energy intensity level of primary energy (MJ/$2021 PPP GDP)</t>
         </is>
       </c>
       <c r="F29" s="9" t="inlineStr">
@@ -7020,7 +7020,7 @@
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Energy intensity level of primary energy (MJ/$2017 PPP GDP)_x</t>
+          <t>Energy intensity level of primary energy (MJ/$2021 PPP GDP)</t>
         </is>
       </c>
       <c r="F45" s="9" t="inlineStr">

</xml_diff>